<commit_message>
Update Campus Connect app
</commit_message>
<xml_diff>
--- a/backend/marks.xlsx
+++ b/backend/marks.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -675,9 +675,101 @@
         <v>8/8/2026, 12:07:09 am</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>pranav</v>
+      </c>
+      <c r="B13" t="str">
+        <v>TE / A</v>
+      </c>
+      <c r="C13" t="str">
+        <v>practical</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Practical-1</v>
+      </c>
+      <c r="E13" t="str">
+        <v>A</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>22/10/2026, 12:11:50 am</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>pranav</v>
+      </c>
+      <c r="B14" t="str">
+        <v>TE / A</v>
+      </c>
+      <c r="C14" t="str">
+        <v>assignment</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Assignment-2</v>
+      </c>
+      <c r="E14" t="str">
+        <v>B</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>22/10/2026, 12:45:01 am</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>pranav</v>
+      </c>
+      <c r="B15" t="str">
+        <v>TE / A</v>
+      </c>
+      <c r="C15" t="str">
+        <v>practical</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Practical-1</v>
+      </c>
+      <c r="E15" t="str">
+        <v>A</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>22/10/2026, 12:45:27 am</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>pranav</v>
+      </c>
+      <c r="B16" t="str">
+        <v>TE / A</v>
+      </c>
+      <c r="C16" t="str">
+        <v>assignment</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Assignment-1</v>
+      </c>
+      <c r="E16" t="str">
+        <v>B</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>22/10/2026, 1:06:28 am</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>